<commit_message>
4.1.5	07/08/2025 Report > Payroll Tax: Revisi data laporan. Penambahan kolom PPH Final, PPH terbayar, PPH Net utk bulan Desember
</commit_message>
<xml_diff>
--- a/system/storage/file/Tax21 Template.xlsx
+++ b/system/storage/file/Tax21 Template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27231"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C872FB8B-8BAA-41AC-8614-B4630D53E13B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C010D582-EB62-4145-B628-8166DDA97E53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>JABATAN</t>
   </si>
@@ -54,10 +54,6 @@
   </si>
   <si>
     <t>GAJI POKOK</t>
-  </si>
-  <si>
-    <t>TOTAL
-TUNJANGAN</t>
   </si>
   <si>
     <t>PENGHASILAN
@@ -87,6 +83,21 @@
   </si>
   <si>
     <t>LAPORAN PPH21</t>
+  </si>
+  <si>
+    <t>TUNJANGAN</t>
+  </si>
+  <si>
+    <t>POTONGAN</t>
+  </si>
+  <si>
+    <t>PPH 21 FINAL</t>
+  </si>
+  <si>
+    <t>PPH 21 TERBAYAR</t>
+  </si>
+  <si>
+    <t>SISA PPH 21</t>
   </si>
 </sst>
 </file>
@@ -248,7 +259,7 @@
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -272,6 +283,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -281,12 +297,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -598,7 +608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:S6"/>
+  <dimension ref="A1:W6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -609,26 +619,26 @@
     <col min="7" max="7" width="6.21875" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
     <col min="9" max="9" width="6.21875" customWidth="1"/>
-    <col min="10" max="13" width="15.109375" customWidth="1"/>
-    <col min="15" max="19" width="15.109375" customWidth="1"/>
+    <col min="10" max="16" width="15.109375" customWidth="1"/>
+    <col min="18" max="23" width="15.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:23" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:19" s="18" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:23" s="15" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B2" s="4"/>
       <c r="F2" s="5">
         <v>46014</v>
       </c>
     </row>
-    <row r="3" spans="1:19" s="1" customFormat="1" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" s="1" customFormat="1" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>5</v>
       </c>
@@ -636,7 +646,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>7</v>
@@ -660,41 +670,53 @@
         <v>12</v>
       </c>
       <c r="K3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="N3" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="L3" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="M3" s="6" t="s">
+      <c r="Q3" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="N3" s="6" t="s">
+      <c r="R3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="O3" s="6" t="s">
+      <c r="S3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="T3" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="U3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="V3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="P3" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q3" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="R3" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="S3" s="6" t="s">
+      <c r="W3" s="6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="19"/>
+      <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -713,29 +735,41 @@
       <c r="M4" s="8">
         <v>0</v>
       </c>
-      <c r="N4" s="12">
-        <v>0</v>
-      </c>
-      <c r="O4" s="17">
+      <c r="N4" s="8">
+        <v>0</v>
+      </c>
+      <c r="O4" s="8">
         <v>0</v>
       </c>
       <c r="P4" s="8">
         <v>0</v>
       </c>
-      <c r="Q4" s="8">
-        <v>0</v>
-      </c>
-      <c r="R4" s="8">
-        <v>0</v>
-      </c>
-      <c r="S4" s="8">
+      <c r="Q4" s="12">
+        <v>0</v>
+      </c>
+      <c r="R4" s="14">
+        <v>0</v>
+      </c>
+      <c r="S4" s="14">
+        <v>0</v>
+      </c>
+      <c r="T4" s="8">
+        <v>0</v>
+      </c>
+      <c r="U4" s="14">
+        <v>0</v>
+      </c>
+      <c r="V4" s="8">
+        <v>0</v>
+      </c>
+      <c r="W4" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
-      <c r="C5" s="19"/>
+      <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -746,35 +780,43 @@
       <c r="K5" s="8"/>
       <c r="L5" s="8"/>
       <c r="M5" s="8"/>
-      <c r="N5" s="12"/>
-      <c r="O5" s="17"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8"/>
       <c r="P5" s="8"/>
-      <c r="Q5" s="8"/>
-      <c r="R5" s="8"/>
-      <c r="S5" s="8"/>
+      <c r="Q5" s="12"/>
+      <c r="R5" s="14"/>
+      <c r="S5" s="14"/>
+      <c r="T5" s="8"/>
+      <c r="U5" s="14"/>
+      <c r="V5" s="8"/>
+      <c r="W5" s="8"/>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A6" s="13" t="s">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A6" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="15"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="18"/>
       <c r="J6" s="9"/>
       <c r="K6" s="9"/>
       <c r="L6" s="9"/>
-      <c r="M6" s="8"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="17"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
       <c r="P6" s="8"/>
-      <c r="Q6" s="8"/>
-      <c r="R6" s="8"/>
+      <c r="Q6" s="3"/>
+      <c r="R6" s="14"/>
       <c r="S6" s="8"/>
+      <c r="T6" s="8"/>
+      <c r="U6" s="8"/>
+      <c r="V6" s="8"/>
+      <c r="W6" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>